<commit_message>
feat: Implementa automação de RPA para lançamentos contábeis
Este commit introduz uma solução completa de automação de processos robóticos (RPA) para o sistema Domínio Contabilidade Fiscal.

A solução inclui:
- Um script otimizado (`rpa.py`) que lê e processa dados de planilhas Excel, utilizando um `config.json` para mapeamento dinâmico de colunas. A leitura é performática, focando apenas nas colunas necessárias.
- Um módulo de automação de interface (`automacao_interface.py`) que utiliza a biblioteca `pywinauto` para preencher os dados lidos na janela de lançamentos do sistema Domínio.
- Funções auxiliares (`utils.py`) para modularizar a lógica de detecção de colunas.
- Documentação completa (`README.md`) e lista de dependências (`requirements.txt`).
- Logging detalhado e tratamento robusto de exceções em todo o processo.
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -425,57 +425,88 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Nome Completo</t>
+          <t>conta a debitar</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>CPF</t>
+          <t>conta a creditar</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Data de Nascimento</t>
+          <t>valor do lancamento</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>descricao</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Jules Verne</t>
+          <t>11101001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>123.456.789-00</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>1828-02-08</t>
+          <t>21101001</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>1500.5</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Pagamento de fornecedor A</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Jane Doe</t>
+          <t>11101002</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>987.654.321-99</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>1990-01-01</t>
+          <t>21101002</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>750</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Adiantamento de salário</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>11101003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>21101003</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>300.25</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Compra de material de escritório</t>
         </is>
       </c>
     </row>

</xml_diff>